<commit_message>
Updated code and data
</commit_message>
<xml_diff>
--- a/Notes and data for listed articles/(row 1) data for 2024 Xu et al. /raw_data/data_for_FC_among_12_ROI.xlsx
+++ b/Notes and data for listed articles/(row 1) data for 2024 Xu et al. /raw_data/data_for_FC_among_12_ROI.xlsx
@@ -192,7 +192,7 @@
     <xdr:ext cx="2762250" cy="2257425"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.png" title="Image"/>
+        <xdr:cNvPr id="0" name="image3.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -220,7 +220,7 @@
     <xdr:ext cx="2762250" cy="1714500"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Image"/>
+        <xdr:cNvPr id="0" name="image1.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -248,7 +248,7 @@
     <xdr:ext cx="2990850" cy="2486025"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.png" title="Image"/>
+        <xdr:cNvPr id="0" name="image4.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -276,7 +276,7 @@
     <xdr:ext cx="2990850" cy="1781175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Image"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>

</xml_diff>